<commit_message>
Tuan09/TH07Kết quả chạy mô hình
</commit_message>
<xml_diff>
--- a/eda/ket_qua/ket_qua_modelNB.xlsx
+++ b/eda/ket_qua/ket_qua_modelNB.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -597,6 +597,32 @@
         <v>120</v>
       </c>
       <c r="H6" t="n">
+        <v>0.567741935483871</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.70995670995671</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.7729559748427673</v>
+      </c>
+      <c r="D7" t="n">
+        <v>44</v>
+      </c>
+      <c r="E7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F7" t="n">
+        <v>37</v>
+      </c>
+      <c r="G7" t="n">
+        <v>120</v>
+      </c>
+      <c r="H7" t="n">
         <v>0.567741935483871</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Tuan09/TH07Update lại cho clean
</commit_message>
<xml_diff>
--- a/eda/ket_qua/ket_qua_modelNB.xlsx
+++ b/eda/ket_qua/ket_qua_modelNB.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,136 +493,6 @@
         <v>120</v>
       </c>
       <c r="H2" t="n">
-        <v>0.567741935483871</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="B3" t="n">
-        <v>0.70995670995671</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.7729559748427673</v>
-      </c>
-      <c r="D3" t="n">
-        <v>44</v>
-      </c>
-      <c r="E3" t="n">
-        <v>30</v>
-      </c>
-      <c r="F3" t="n">
-        <v>37</v>
-      </c>
-      <c r="G3" t="n">
-        <v>120</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.567741935483871</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.70995670995671</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.7729559748427673</v>
-      </c>
-      <c r="D4" t="n">
-        <v>44</v>
-      </c>
-      <c r="E4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F4" t="n">
-        <v>37</v>
-      </c>
-      <c r="G4" t="n">
-        <v>120</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.567741935483871</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="B5" t="n">
-        <v>0.70995670995671</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.7729559748427673</v>
-      </c>
-      <c r="D5" t="n">
-        <v>44</v>
-      </c>
-      <c r="E5" t="n">
-        <v>30</v>
-      </c>
-      <c r="F5" t="n">
-        <v>37</v>
-      </c>
-      <c r="G5" t="n">
-        <v>120</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.567741935483871</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="B6" t="n">
-        <v>0.70995670995671</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.7729559748427673</v>
-      </c>
-      <c r="D6" t="n">
-        <v>44</v>
-      </c>
-      <c r="E6" t="n">
-        <v>30</v>
-      </c>
-      <c r="F6" t="n">
-        <v>37</v>
-      </c>
-      <c r="G6" t="n">
-        <v>120</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.567741935483871</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="B7" t="n">
-        <v>0.70995670995671</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.7729559748427673</v>
-      </c>
-      <c r="D7" t="n">
-        <v>44</v>
-      </c>
-      <c r="E7" t="n">
-        <v>30</v>
-      </c>
-      <c r="F7" t="n">
-        <v>37</v>
-      </c>
-      <c r="G7" t="n">
-        <v>120</v>
-      </c>
-      <c r="H7" t="n">
         <v>0.567741935483871</v>
       </c>
     </row>

</xml_diff>